<commit_message>
Update example data including an 'inf' value
</commit_message>
<xml_diff>
--- a/mibiscreen/data/example_data/example_data.xlsx
+++ b/mibiscreen/data/example_data/example_data.xlsx
@@ -5,13 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="contaminants" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="environment" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="metabolites" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="isotopes" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="contaminants" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="environment" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="metabolites" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="isotopes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="46">
   <si>
     <t xml:space="preserve">sample_nr</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t xml:space="preserve">ug/l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inf</t>
   </si>
   <si>
     <t xml:space="preserve">delta_13C-benzene</t>
@@ -215,8 +218,8 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <name val=""/>
-      <family val="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -277,32 +280,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -318,8 +325,114 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -548,14 +661,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P6"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1017" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1017" style="3" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -609,252 +722,252 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="M2" s="0" t="s">
+      <c r="M2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N2" s="0" t="s">
+      <c r="N2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="O2" s="0" t="s">
+      <c r="O2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="P2" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="3" t="n">
         <v>-12</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="3" t="n">
         <v>7.23</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="3" t="n">
         <v>322</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="3" t="n">
         <v>-208</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="3" t="n">
         <v>0.3</v>
       </c>
-      <c r="H3" s="0" t="n">
+      <c r="H3" s="3" t="n">
         <v>122</v>
       </c>
-      <c r="I3" s="0" t="n">
+      <c r="I3" s="3" t="n">
         <v>0.58</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="K3" s="0" t="n">
+      <c r="K3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="0" t="n">
+      <c r="L3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3" t="n">
         <v>748</v>
       </c>
-      <c r="N3" s="0" t="n">
+      <c r="N3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="O3" s="0" t="n">
+      <c r="O3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P3" s="0" t="n">
+      <c r="P3" s="3" t="n">
         <v>1.6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="3" t="n">
         <v>-15.5</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="3" t="n">
         <v>7.67</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="3" t="n">
         <v>405</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="3" t="n">
         <v>-231</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H4" s="0" t="n">
+      <c r="H4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="0" t="n">
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="L4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="0" t="n">
+      <c r="L4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="N4" s="0" t="n">
+      <c r="N4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="0" t="n">
+      <c r="O4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="3" t="n">
         <v>-17</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="3" t="n">
         <v>7.75</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="3" t="n">
         <v>223</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="3" t="n">
         <v>-252</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="0" t="n">
+      <c r="I5" s="3" t="n">
         <v>0.03</v>
       </c>
-      <c r="J5" s="0" t="n">
+      <c r="J5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K5" s="0" t="n">
+      <c r="K5" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="0" t="n">
+      <c r="L5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="N5" s="0" t="n">
+      <c r="N5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="0" t="n">
+      <c r="O5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="3" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="3" t="n">
         <v>-19</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="3" t="n">
         <v>7.53</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="3" t="n">
         <v>-317</v>
       </c>
-      <c r="G6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="0" t="n">
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>180</v>
       </c>
-      <c r="I6" s="0" t="n">
+      <c r="I6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="0" t="n">
+      <c r="J6" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="K6" s="0" t="n">
+      <c r="K6" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="L6" s="0" t="n">
+      <c r="L6" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="M6" s="0" t="n">
+      <c r="M6" s="3" t="n">
         <v>122</v>
       </c>
-      <c r="N6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="0" t="n">
+      <c r="N6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="3" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -863,43 +976,43 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="8.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="5.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="3" width="8.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="5.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="10.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="9.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>40</v>
       </c>
     </row>
@@ -913,13 +1026,13 @@
       <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="3" t="s">
         <v>41</v>
       </c>
     </row>
@@ -933,13 +1046,13 @@
       <c r="C3" s="2" t="n">
         <v>-12</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="3" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="3" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -953,10 +1066,10 @@
       <c r="C4" s="2" t="n">
         <v>-15.5</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="0" t="n">
+      <c r="E4" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F4" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -970,13 +1083,13 @@
       <c r="C5" s="2" t="n">
         <v>-17</v>
       </c>
-      <c r="D5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="0" t="n">
+      <c r="D5" s="3" t="n">
         <v>11.4</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="E5" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="3" t="n">
         <v>5.4</v>
       </c>
     </row>
@@ -990,13 +1103,13 @@
       <c r="C6" s="2" t="n">
         <v>-19</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="3" t="n">
         <v>0.3</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="3" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -1005,40 +1118,40 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="8.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="3" width="8.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="13.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="12.71"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
+    <row r="1" s="7" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>43</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1051,11 +1164,11 @@
       <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>44</v>
+      <c r="D2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1068,10 +1181,10 @@
       <c r="C3" s="2" t="n">
         <v>-12</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="3" t="n">
         <v>-26.1</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="3" t="n">
         <v>-106</v>
       </c>
     </row>
@@ -1085,10 +1198,10 @@
       <c r="C4" s="2" t="n">
         <v>-15.5</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="3" t="n">
         <v>-25.8</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="3" t="n">
         <v>-110</v>
       </c>
     </row>
@@ -1102,10 +1215,10 @@
       <c r="C5" s="2" t="n">
         <v>-17</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="3" t="n">
         <v>-24.1</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="3" t="n">
         <v>-118</v>
       </c>
     </row>
@@ -1119,10 +1232,10 @@
       <c r="C6" s="2" t="n">
         <v>-19</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="3" t="n">
         <v>-24.1</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="3" t="n">
         <v>-117</v>
       </c>
     </row>
@@ -1131,8 +1244,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>